<commit_message>
fix: A-levels after audit - Imperial Aero recommends Further Mathematics (12 -> 13), Manchester counted as Mathematics compulsory (20), one named/compulsory vocabulary in The Unfashionable Four, Cambridge CS as the page puts it, US paragraph, Dataset JSON-LD without 2025, old 31-programme wording on the hub and three articles, viz/04 removed
</commit_message>
<xml_diff>
--- a/research/long-bet/raw/ALevel_Prerequisites.xlsx
+++ b/research/long-bet/raw/ALevel_Prerequisites.xlsx
@@ -1611,7 +1611,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Further Mathematics</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2350,10 +2350,10 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Actuarial Science; Applied Mathematics; Chemical Engineering; Chemistry; Computer Science; Data Science; Earth Sciences; Electrical Engineering; Engineering (General); Materials Science; Physics; Statistics</t>
+          <t>Actuarial Science; Aerospace Engineering; Applied Mathematics; Chemical Engineering; Chemistry; Computer Science; Data Science; Earth Sciences; Electrical Engineering; Engineering (General); Materials Science; Physics; Statistics</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: audit 2 closing - Manchester rule referenced in Limitations, n_required 0 for Civil, four outside the cluster, condensed version wording on marketing-market
</commit_message>
<xml_diff>
--- a/research/long-bet/raw/ALevel_Prerequisites.xlsx
+++ b/research/long-bet/raw/ALevel_Prerequisites.xlsx
@@ -1468,7 +1468,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>—</t>

</xml_diff>